<commit_message>
edicion de bugs por PARA subida de datos en la base de datos BI y creacion de .xlsx
</commit_message>
<xml_diff>
--- a/inventario.xlsx
+++ b/inventario.xlsx
@@ -461,7 +461,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="str">
@@ -470,37 +470,77 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="str">
-        <v>Facturación</v>
+        <v>TECNOLOGÍAS DE LA INFORMACIÓN</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="str">
-        <v>Busness Inteligence</v>
+        <v>RECURSOS HUMANOS</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="str">
-        <v>Cuentas Por Cobrar</v>
+        <v>CALIDAD, SEGURIDAD, SALUD Y MEDIO AMBIENTE</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="str">
-        <v>Cuentas Por Pagar</v>
+        <v>INFRAESTRUCTURA Y CIBERSEGURIDAD</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="str">
-        <v>Compras</v>
+        <v>BUSINESS INTELLIGENCE</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="str">
-        <v>Administración</v>
+        <v>OPERACIONES VERACRUZ</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="str">
+        <v>ATENCION A CLIENTES</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="str">
+        <v>INVESTIGACIÓN CLINICA</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="str">
+        <v>NORMATIVIDAD</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="str">
+        <v>OPERACIONES AICM Y AIFA</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="str">
+        <v>TESORERIA</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="str">
+        <v>CONTABILIDAD</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="str">
+        <v>ADMINISTRACIÓN</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="str">
+        <v>CONTRALORIA</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
edicion de inventario.xlsx para las areas de cada equipo
</commit_message>
<xml_diff>
--- a/inventario.xlsx
+++ b/inventario.xlsx
@@ -461,7 +461,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A32"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="str">
@@ -538,9 +538,94 @@
         <v>CONTRALORIA</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="1" t="str">
+        <v>COMPRAS</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="str">
+        <v>CUENTAS POR PAGAR</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="str">
+        <v>CUENTAS POR COBRAR</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="str">
+        <v>CONTABILIDAD ABC</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="str">
+        <v>CONTABILIDAD SEC</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="str">
+        <v>FACTURACIÓN SEC</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="str">
+        <v>FACTURACIÓN ABC</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="str">
+        <v>LEGAL</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="str">
+        <v>OPERACIONES Y LOGÍSTICA</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="str">
+        <v>AYUDANTE GENERAL</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="str">
+        <v>MENSAJERO</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="str">
+        <v>OPERADORES</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="str">
+        <v>GLOSA</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="str">
+        <v>OPERACIONES</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="str">
+        <v>ATENCIÓN A CLIENTES</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="str">
+        <v>MESA DE CONTROL</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="str">
+        <v>PROSPECCIÓN DE NEGOCIOS</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A32"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>